<commit_message>
paper run 2026-10-23 16:48
</commit_message>
<xml_diff>
--- a/reports/2026-10-23.xlsx
+++ b/reports/2026-10-23.xlsx
@@ -614,7 +614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -767,13 +767,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C15" t="n">
         <v>6</v>
       </c>
       <c r="D15" t="n">
-        <v>970.46</v>
+        <v>764.38</v>
       </c>
       <c r="E15" t="n">
         <v>303.6</v>
@@ -782,52 +782,52 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>По активам</t>
-        </is>
+          <t>5m</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" t="n">
+        <v>159.93</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>BTC</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>3</v>
-      </c>
-      <c r="C17" t="n">
-        <v>3</v>
-      </c>
-      <c r="D17" t="n">
-        <v>500.51</v>
-      </c>
-      <c r="E17" t="n">
-        <v>253.19</v>
+          <t>По активам</t>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ETH</t>
+          <t>BTC</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C18" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D18" t="n">
-        <v>108.91</v>
+        <v>500.51</v>
       </c>
       <c r="E18" t="n">
-        <v>0</v>
+        <v>253.19</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SOL</t>
+          <t>ETH</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -837,116 +837,116 @@
         <v>1</v>
       </c>
       <c r="D19" t="n">
-        <v>180.52</v>
+        <v>108.91</v>
       </c>
       <c r="E19" t="n">
-        <v>50.41</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>XRP</t>
+          <t>SOL</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C20" t="n">
         <v>1</v>
       </c>
       <c r="D20" t="n">
-        <v>180.52</v>
+        <v>-25.56</v>
       </c>
       <c r="E20" t="n">
-        <v>0</v>
+        <v>50.41</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>2</v>
+      </c>
+      <c r="C21" t="n">
+        <v>2</v>
+      </c>
+      <c r="D21" t="n">
+        <v>340.45</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>5</v>
-      </c>
-      <c r="C22" t="n">
-        <v>5</v>
-      </c>
-      <c r="D22" t="n">
-        <v>861.55</v>
-      </c>
-      <c r="E22" t="n">
-        <v>303.6</v>
+          <t>По цене входа</t>
+        </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0.60–0.62</t>
+          <t>0.50–0.55</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C23" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D23" t="n">
-        <v>108.91</v>
+        <v>815.4</v>
       </c>
       <c r="E23" t="n">
-        <v>0</v>
+        <v>303.6</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>По риск-гейтам</t>
-        </is>
+          <t>0.60–0.62</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>1</v>
+      </c>
+      <c r="C24" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" t="n">
+        <v>108.91</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>MAX_PER_WINDOW</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>2</v>
-      </c>
-      <c r="C25" t="n">
-        <v>2</v>
-      </c>
-      <c r="D25" t="n">
-        <v>289.43</v>
-      </c>
-      <c r="E25" t="n">
-        <v>0</v>
+          <t>По риск-гейтам</t>
+        </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>NO_LIQUIDITY</t>
+          <t>MAX_PER_WINDOW</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D26" t="n">
-        <v>160.77</v>
+        <v>289.43</v>
       </c>
       <c r="E26" t="n">
         <v>0</v>
@@ -955,302 +955,321 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>NO_LIQUIDITY</t>
         </is>
       </c>
       <c r="B27" t="n">
         <v>3</v>
       </c>
       <c r="C27" t="n">
+        <v>2</v>
+      </c>
+      <c r="D27" t="n">
+        <v>114.62</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
         <v>3</v>
       </c>
-      <c r="D27" t="n">
+      <c r="C28" t="n">
+        <v>3</v>
+      </c>
+      <c r="D28" t="n">
         <v>520.26</v>
       </c>
-      <c r="E27" t="n">
+      <c r="E28" t="n">
         <v>303.6</v>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
+    <row r="30">
+      <c r="A30" t="inlineStr">
         <is>
           <t>REALIZED (реальные сделки)</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>По активам</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>BTC</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
-        <v>2</v>
-      </c>
-      <c r="C32" t="n">
-        <v>2</v>
-      </c>
-      <c r="D32" t="n">
-        <v>253.19</v>
+          <t>По активам</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>2</v>
+      </c>
+      <c r="C33" t="n">
+        <v>2</v>
+      </c>
+      <c r="D33" t="n">
+        <v>253.19</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
           <t>SOL</t>
         </is>
       </c>
-      <c r="B33" t="n">
-        <v>1</v>
-      </c>
-      <c r="C33" t="n">
-        <v>1</v>
-      </c>
-      <c r="D33" t="n">
+      <c r="B34" t="n">
+        <v>1</v>
+      </c>
+      <c r="C34" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" t="n">
         <v>50.41</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>По окнам</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
+          <t>По окнам</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
           <t>15m</t>
         </is>
       </c>
-      <c r="B36" t="n">
+      <c r="B37" t="n">
         <v>3</v>
       </c>
-      <c r="C36" t="n">
+      <c r="C37" t="n">
         <v>3</v>
       </c>
-      <c r="D36" t="n">
+      <c r="D37" t="n">
         <v>303.6</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>По часам</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
+          <t>По часам</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
           <t>01</t>
         </is>
       </c>
-      <c r="B39" t="n">
+      <c r="B40" t="n">
         <v>3</v>
       </c>
-      <c r="C39" t="n">
+      <c r="C40" t="n">
         <v>3</v>
       </c>
-      <c r="D39" t="n">
+      <c r="D40" t="n">
         <v>303.6</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
           <t>0.50–0.55</t>
         </is>
       </c>
-      <c r="B42" t="n">
+      <c r="B43" t="n">
         <v>3</v>
       </c>
-      <c r="C42" t="n">
+      <c r="C43" t="n">
         <v>3</v>
       </c>
-      <c r="D42" t="n">
+      <c r="D43" t="n">
         <v>303.6</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>По силе движения</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>0.10–0.12%</t>
-        </is>
-      </c>
-      <c r="B45" t="n">
-        <v>2</v>
-      </c>
-      <c r="C45" t="n">
-        <v>2</v>
-      </c>
-      <c r="D45" t="n">
-        <v>253.19</v>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
+          <t>0.10–0.12%</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>2</v>
+      </c>
+      <c r="C46" t="n">
+        <v>2</v>
+      </c>
+      <c r="D46" t="n">
+        <v>253.19</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
           <t>0.15–0.20%</t>
         </is>
       </c>
-      <c r="B46" t="n">
-        <v>1</v>
-      </c>
-      <c r="C46" t="n">
-        <v>1</v>
-      </c>
-      <c r="D46" t="n">
+      <c r="B47" t="n">
+        <v>1</v>
+      </c>
+      <c r="C47" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" t="n">
         <v>50.41</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>По направлению</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="B49" t="n">
-        <v>2</v>
-      </c>
-      <c r="C49" t="n">
-        <v>2</v>
-      </c>
-      <c r="D49" t="n">
-        <v>216.2</v>
+          <t>По направлению</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>2</v>
+      </c>
+      <c r="C50" t="n">
+        <v>2</v>
+      </c>
+      <c r="D50" t="n">
+        <v>216.2</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
           <t>UP</t>
         </is>
       </c>
-      <c r="B50" t="n">
-        <v>1</v>
-      </c>
-      <c r="C50" t="n">
-        <v>1</v>
-      </c>
-      <c r="D50" t="n">
+      <c r="B51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C51" t="n">
+        <v>1</v>
+      </c>
+      <c r="D51" t="n">
         <v>87.40000000000001</v>
       </c>
     </row>

</xml_diff>

<commit_message>
paper run 2026-10-23 22:28
</commit_message>
<xml_diff>
--- a/reports/2026-10-23.xlsx
+++ b/reports/2026-10-23.xlsx
@@ -767,13 +767,13 @@
         </is>
       </c>
       <c r="B15" t="n">
+        <v>8</v>
+      </c>
+      <c r="C15" t="n">
         <v>7</v>
       </c>
-      <c r="C15" t="n">
-        <v>6</v>
-      </c>
       <c r="D15" t="n">
-        <v>764.38</v>
+        <v>939.9299999999999</v>
       </c>
       <c r="E15" t="n">
         <v>303.6</v>
@@ -786,13 +786,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D16" t="n">
-        <v>159.93</v>
+        <v>290.42</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -869,13 +869,13 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D21" t="n">
-        <v>340.45</v>
+        <v>646.49</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
@@ -895,13 +895,13 @@
         </is>
       </c>
       <c r="B23" t="n">
+        <v>8</v>
+      </c>
+      <c r="C23" t="n">
         <v>7</v>
       </c>
-      <c r="C23" t="n">
-        <v>6</v>
-      </c>
       <c r="D23" t="n">
-        <v>815.4</v>
+        <v>990.95</v>
       </c>
       <c r="E23" t="n">
         <v>303.6</v>
@@ -914,13 +914,13 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D24" t="n">
-        <v>108.91</v>
+        <v>239.4</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
@@ -959,13 +959,13 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C27" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D27" t="n">
-        <v>114.62</v>
+        <v>420.66</v>
       </c>
       <c r="E27" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
paper run 2026-10-24 04:09
</commit_message>
<xml_diff>
--- a/reports/2026-10-23.xlsx
+++ b/reports/2026-10-23.xlsx
@@ -767,13 +767,13 @@
         </is>
       </c>
       <c r="B15" t="n">
+        <v>9</v>
+      </c>
+      <c r="C15" t="n">
         <v>8</v>
       </c>
-      <c r="C15" t="n">
-        <v>7</v>
-      </c>
       <c r="D15" t="n">
-        <v>939.9299999999999</v>
+        <v>1097.68</v>
       </c>
       <c r="E15" t="n">
         <v>303.6</v>
@@ -869,13 +869,13 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C21" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D21" t="n">
-        <v>646.49</v>
+        <v>804.24</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
@@ -895,13 +895,13 @@
         </is>
       </c>
       <c r="B23" t="n">
+        <v>9</v>
+      </c>
+      <c r="C23" t="n">
         <v>8</v>
       </c>
-      <c r="C23" t="n">
-        <v>7</v>
-      </c>
       <c r="D23" t="n">
-        <v>990.95</v>
+        <v>1148.7</v>
       </c>
       <c r="E23" t="n">
         <v>303.6</v>
@@ -959,13 +959,13 @@
         </is>
       </c>
       <c r="B27" t="n">
+        <v>6</v>
+      </c>
+      <c r="C27" t="n">
         <v>5</v>
       </c>
-      <c r="C27" t="n">
-        <v>4</v>
-      </c>
       <c r="D27" t="n">
-        <v>420.66</v>
+        <v>578.41</v>
       </c>
       <c r="E27" t="n">
         <v>0</v>

</xml_diff>